<commit_message>
Update September daily routine
</commit_message>
<xml_diff>
--- a/12623065.xlsx
+++ b/12623065.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -265,6 +265,63 @@
   </si>
   <si>
     <t>Good use of time.</t>
+  </si>
+  <si>
+    <t>Felt satisfied with my progress.</t>
+  </si>
+  <si>
+    <t>completed my classes and stayed on schedule.</t>
+  </si>
+  <si>
+    <t>Good day with regular classes.</t>
+  </si>
+  <si>
+    <t>Had a good day and manage my time well.</t>
+  </si>
+  <si>
+    <t>Started the week with a focused.</t>
+  </si>
+  <si>
+    <t>Attend all classes.</t>
+  </si>
+  <si>
+    <t>Made good use of my time.</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Fresher's party is organized today.Enjoying with friends but feeling low .</t>
+  </si>
+  <si>
+    <t>Ending the day with satisfaction.</t>
+  </si>
+  <si>
+    <t>Relaxing and preparing for upcoming week.</t>
+  </si>
+  <si>
+    <t>Focusing more on studies.</t>
+  </si>
+  <si>
+    <t>Keeping myself motivated.</t>
+  </si>
+  <si>
+    <t>Mainting the schedule.</t>
+  </si>
+  <si>
+    <t>Feeling a little tired.</t>
+  </si>
+  <si>
+    <t>Working hard on my work.</t>
+  </si>
+  <si>
+    <t>Preparing for CA.</t>
+  </si>
+  <si>
+    <t>Today I had my CA , and it went very well.So feeling good.</t>
   </si>
 </sst>
 </file>
@@ -985,7 +1042,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1022,6 +1079,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1359,181 +1431,181 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25" spans="1:1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" ht="16.5" spans="1:1">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="23" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="19"/>
+      <c r="A4" s="24"/>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="25" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="24" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="19"/>
+      <c r="A7" s="24"/>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="24" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="24" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="24" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" s="19"/>
+      <c r="A12" s="24"/>
     </row>
     <row r="13" spans="1:1">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="25" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:1">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="24" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:1">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="24" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:1">
-      <c r="A16" s="19"/>
+      <c r="A16" s="24"/>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="24" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="24" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="24" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="24" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="24" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="24" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="24" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="24" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="24" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="24" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="24" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="24" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="24" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="19"/>
+      <c r="A32" s="24"/>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="25" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="24" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="24" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="19"/>
+      <c r="A36" s="24"/>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="20"/>
+      <c r="A37" s="25"/>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="19"/>
+      <c r="A38" s="24"/>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="19"/>
+      <c r="A39" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2731,327 +2803,877 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="13"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="15"/>
-    </row>
-    <row r="30" spans="1:14">
-      <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="13"/>
-      <c r="J30" s="13"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-      <c r="N30" s="15"/>
+    <row r="29" ht="30" spans="1:14">
+      <c r="A29" s="16">
+        <v>46266</v>
+      </c>
+      <c r="B29" s="17">
+        <v>420</v>
+      </c>
+      <c r="C29" s="17">
+        <v>20</v>
+      </c>
+      <c r="D29" s="17">
+        <v>120</v>
+      </c>
+      <c r="E29" s="17">
+        <v>40</v>
+      </c>
+      <c r="F29" s="17">
+        <v>300</v>
+      </c>
+      <c r="G29" s="17">
+        <v>6</v>
+      </c>
+      <c r="H29" s="17">
+        <v>30</v>
+      </c>
+      <c r="I29" s="18">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J29" s="18">
+        <f t="shared" si="1"/>
+        <v>510</v>
+      </c>
+      <c r="K29" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L29" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M29" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N29" s="20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" ht="30" spans="1:14">
+      <c r="A30" s="16">
+        <v>46267</v>
+      </c>
+      <c r="B30" s="17">
+        <v>420</v>
+      </c>
+      <c r="C30" s="17">
+        <v>20</v>
+      </c>
+      <c r="D30" s="17">
+        <v>180</v>
+      </c>
+      <c r="E30" s="17">
+        <v>40</v>
+      </c>
+      <c r="F30" s="17">
+        <v>300</v>
+      </c>
+      <c r="G30" s="17">
+        <v>6</v>
+      </c>
+      <c r="H30" s="17">
+        <v>30</v>
+      </c>
+      <c r="I30" s="18">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J30" s="18">
+        <f t="shared" si="1"/>
+        <v>450</v>
+      </c>
+      <c r="K30" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L30" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M30" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N30" s="20" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="31" spans="1:14">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="15"/>
+      <c r="A31" s="16">
+        <v>46268</v>
+      </c>
+      <c r="B31" s="17">
+        <v>420</v>
+      </c>
+      <c r="C31" s="17">
+        <v>20</v>
+      </c>
+      <c r="D31" s="17">
+        <v>180</v>
+      </c>
+      <c r="E31" s="17">
+        <v>40</v>
+      </c>
+      <c r="F31" s="17">
+        <v>200</v>
+      </c>
+      <c r="G31" s="17">
+        <v>4</v>
+      </c>
+      <c r="H31" s="17">
+        <v>50</v>
+      </c>
+      <c r="I31" s="18">
+        <f t="shared" si="0"/>
+        <v>910</v>
+      </c>
+      <c r="J31" s="18">
+        <f t="shared" si="1"/>
+        <v>530</v>
+      </c>
+      <c r="K31" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L31" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M31" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N31" s="20" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="32" spans="1:14">
-      <c r="A32" s="11"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="15"/>
+      <c r="A32" s="16">
+        <v>46269</v>
+      </c>
+      <c r="B32" s="17">
+        <v>420</v>
+      </c>
+      <c r="C32" s="17">
+        <v>20</v>
+      </c>
+      <c r="D32" s="17">
+        <v>180</v>
+      </c>
+      <c r="E32" s="17">
+        <v>30</v>
+      </c>
+      <c r="F32" s="17">
+        <v>250</v>
+      </c>
+      <c r="G32" s="17">
+        <v>5</v>
+      </c>
+      <c r="H32" s="17">
+        <v>40</v>
+      </c>
+      <c r="I32" s="18">
+        <f t="shared" si="0"/>
+        <v>940</v>
+      </c>
+      <c r="J32" s="18">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="K32" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L32" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M32" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N32" s="20"/>
     </row>
     <row r="33" spans="1:14">
-      <c r="A33" s="11"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="15"/>
-    </row>
-    <row r="34" spans="1:14">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="14"/>
-      <c r="N34" s="15"/>
-    </row>
-    <row r="35" spans="1:14">
-      <c r="A35" s="11"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="14"/>
-      <c r="M35" s="14"/>
-      <c r="N35" s="15"/>
+      <c r="A33" s="16">
+        <v>46270</v>
+      </c>
+      <c r="B33" s="17">
+        <v>480</v>
+      </c>
+      <c r="C33" s="17">
+        <v>40</v>
+      </c>
+      <c r="D33" s="17">
+        <v>360</v>
+      </c>
+      <c r="E33" s="17">
+        <v>180</v>
+      </c>
+      <c r="F33" s="17">
+        <v>0</v>
+      </c>
+      <c r="G33" s="17">
+        <v>0</v>
+      </c>
+      <c r="H33" s="17">
+        <v>120</v>
+      </c>
+      <c r="I33" s="18">
+        <f t="shared" si="0"/>
+        <v>1180</v>
+      </c>
+      <c r="J33" s="18">
+        <f t="shared" si="1"/>
+        <v>260</v>
+      </c>
+      <c r="K33" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L33" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M33" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N33" s="20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" ht="30" spans="1:14">
+      <c r="A34" s="16">
+        <v>46271</v>
+      </c>
+      <c r="B34" s="17">
+        <v>480</v>
+      </c>
+      <c r="C34" s="17">
+        <v>60</v>
+      </c>
+      <c r="D34" s="17">
+        <v>240</v>
+      </c>
+      <c r="E34" s="17">
+        <v>120</v>
+      </c>
+      <c r="F34" s="17">
+        <v>0</v>
+      </c>
+      <c r="G34" s="17">
+        <v>0</v>
+      </c>
+      <c r="H34" s="17">
+        <v>50</v>
+      </c>
+      <c r="I34" s="18">
+        <f t="shared" si="0"/>
+        <v>950</v>
+      </c>
+      <c r="J34" s="18">
+        <f t="shared" si="1"/>
+        <v>490</v>
+      </c>
+      <c r="K34" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L34" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M34" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N34" s="20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" ht="30" spans="1:14">
+      <c r="A35" s="16">
+        <v>46272</v>
+      </c>
+      <c r="B35" s="17">
+        <v>420</v>
+      </c>
+      <c r="C35" s="17">
+        <v>20</v>
+      </c>
+      <c r="D35" s="17">
+        <v>120</v>
+      </c>
+      <c r="E35" s="17">
+        <v>40</v>
+      </c>
+      <c r="F35" s="17">
+        <v>300</v>
+      </c>
+      <c r="G35" s="17">
+        <v>6</v>
+      </c>
+      <c r="H35" s="17">
+        <v>30</v>
+      </c>
+      <c r="I35" s="18">
+        <f t="shared" si="0"/>
+        <v>930</v>
+      </c>
+      <c r="J35" s="18">
+        <f t="shared" si="1"/>
+        <v>510</v>
+      </c>
+      <c r="K35" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L35" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M35" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N35" s="20" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="36" spans="1:14">
-      <c r="A36" s="11"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="14"/>
-      <c r="L36" s="14"/>
-      <c r="M36" s="14"/>
-      <c r="N36" s="15"/>
+      <c r="A36" s="16">
+        <v>46273</v>
+      </c>
+      <c r="B36" s="17">
+        <v>420</v>
+      </c>
+      <c r="C36" s="17">
+        <v>20</v>
+      </c>
+      <c r="D36" s="17">
+        <v>120</v>
+      </c>
+      <c r="E36" s="17">
+        <v>40</v>
+      </c>
+      <c r="F36" s="17">
+        <v>300</v>
+      </c>
+      <c r="G36" s="17">
+        <v>6</v>
+      </c>
+      <c r="H36" s="17">
+        <v>20</v>
+      </c>
+      <c r="I36" s="18">
+        <f t="shared" si="0"/>
+        <v>920</v>
+      </c>
+      <c r="J36" s="18">
+        <f t="shared" si="1"/>
+        <v>520</v>
+      </c>
+      <c r="K36" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L36" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M36" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N36" s="20" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="37" spans="1:14">
-      <c r="A37" s="11"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="13"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-      <c r="N37" s="15"/>
-    </row>
-    <row r="38" spans="1:14">
-      <c r="A38" s="11"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="14"/>
-      <c r="L38" s="14"/>
-      <c r="M38" s="14"/>
-      <c r="N38" s="15"/>
-    </row>
-    <row r="39" spans="1:14">
-      <c r="A39" s="11"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="14"/>
-      <c r="L39" s="14"/>
-      <c r="M39" s="14"/>
-      <c r="N39" s="15"/>
-    </row>
-    <row r="40" spans="1:14">
-      <c r="A40" s="11"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="14"/>
-      <c r="L40" s="14"/>
-      <c r="M40" s="14"/>
-      <c r="N40" s="15"/>
+      <c r="A37" s="16">
+        <v>46274</v>
+      </c>
+      <c r="B37" s="17">
+        <v>420</v>
+      </c>
+      <c r="C37" s="17">
+        <v>20</v>
+      </c>
+      <c r="D37" s="17">
+        <v>180</v>
+      </c>
+      <c r="E37" s="17">
+        <v>50</v>
+      </c>
+      <c r="F37" s="17">
+        <v>300</v>
+      </c>
+      <c r="G37" s="17">
+        <v>6</v>
+      </c>
+      <c r="H37" s="17">
+        <v>20</v>
+      </c>
+      <c r="I37" s="18">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J37" s="18">
+        <f t="shared" si="1"/>
+        <v>450</v>
+      </c>
+      <c r="K37" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L37" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M37" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N37" s="20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" ht="45" spans="1:14">
+      <c r="A38" s="16">
+        <v>46275</v>
+      </c>
+      <c r="B38" s="17">
+        <v>420</v>
+      </c>
+      <c r="C38" s="17">
+        <v>30</v>
+      </c>
+      <c r="D38" s="17">
+        <v>60</v>
+      </c>
+      <c r="E38" s="17">
+        <v>20</v>
+      </c>
+      <c r="F38" s="17">
+        <v>100</v>
+      </c>
+      <c r="G38" s="17">
+        <v>2</v>
+      </c>
+      <c r="H38" s="17">
+        <v>180</v>
+      </c>
+      <c r="I38" s="18">
+        <f t="shared" si="0"/>
+        <v>810</v>
+      </c>
+      <c r="J38" s="18">
+        <f t="shared" si="1"/>
+        <v>630</v>
+      </c>
+      <c r="K38" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="L38" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M38" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="N38" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" ht="30" spans="1:14">
+      <c r="A39" s="16">
+        <v>46276</v>
+      </c>
+      <c r="B39" s="17">
+        <v>420</v>
+      </c>
+      <c r="C39" s="17">
+        <v>30</v>
+      </c>
+      <c r="D39" s="17">
+        <v>120</v>
+      </c>
+      <c r="E39" s="17">
+        <v>60</v>
+      </c>
+      <c r="F39" s="17">
+        <v>250</v>
+      </c>
+      <c r="G39" s="17">
+        <v>5</v>
+      </c>
+      <c r="H39" s="17">
+        <v>30</v>
+      </c>
+      <c r="I39" s="18">
+        <f t="shared" si="0"/>
+        <v>910</v>
+      </c>
+      <c r="J39" s="18">
+        <f t="shared" si="1"/>
+        <v>530</v>
+      </c>
+      <c r="K39" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L39" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M39" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N39" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" ht="30" spans="1:14">
+      <c r="A40" s="16">
+        <v>46277</v>
+      </c>
+      <c r="B40" s="17">
+        <v>480</v>
+      </c>
+      <c r="C40" s="17">
+        <v>30</v>
+      </c>
+      <c r="D40" s="17">
+        <v>240</v>
+      </c>
+      <c r="E40" s="17">
+        <v>60</v>
+      </c>
+      <c r="F40" s="17">
+        <v>0</v>
+      </c>
+      <c r="G40" s="17">
+        <v>0</v>
+      </c>
+      <c r="H40" s="17">
+        <v>60</v>
+      </c>
+      <c r="I40" s="18">
+        <f t="shared" si="0"/>
+        <v>870</v>
+      </c>
+      <c r="J40" s="18">
+        <f t="shared" si="1"/>
+        <v>570</v>
+      </c>
+      <c r="K40" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L40" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M40" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N40" s="20" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="41" spans="1:14">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="14"/>
-      <c r="L41" s="14"/>
-      <c r="M41" s="14"/>
-      <c r="N41" s="15"/>
+      <c r="A41" s="16">
+        <v>46278</v>
+      </c>
+      <c r="B41" s="17">
+        <v>480</v>
+      </c>
+      <c r="C41" s="17">
+        <v>40</v>
+      </c>
+      <c r="D41" s="17">
+        <v>360</v>
+      </c>
+      <c r="E41" s="17">
+        <v>50</v>
+      </c>
+      <c r="F41" s="17">
+        <v>0</v>
+      </c>
+      <c r="G41" s="17">
+        <v>0</v>
+      </c>
+      <c r="H41" s="17">
+        <v>90</v>
+      </c>
+      <c r="I41" s="18">
+        <f t="shared" si="0"/>
+        <v>1020</v>
+      </c>
+      <c r="J41" s="18">
+        <f t="shared" si="1"/>
+        <v>420</v>
+      </c>
+      <c r="K41" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L41" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M41" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N41" s="20" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="42" spans="1:14">
-      <c r="A42" s="11"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="13"/>
-      <c r="K42" s="14"/>
-      <c r="L42" s="14"/>
-      <c r="M42" s="14"/>
-      <c r="N42" s="15"/>
+      <c r="A42" s="16">
+        <v>46279</v>
+      </c>
+      <c r="B42" s="17">
+        <v>420</v>
+      </c>
+      <c r="C42" s="17">
+        <v>20</v>
+      </c>
+      <c r="D42" s="17">
+        <v>180</v>
+      </c>
+      <c r="E42" s="17">
+        <v>40</v>
+      </c>
+      <c r="F42" s="17">
+        <v>300</v>
+      </c>
+      <c r="G42" s="17">
+        <v>6</v>
+      </c>
+      <c r="H42" s="17">
+        <v>150</v>
+      </c>
+      <c r="I42" s="18">
+        <f t="shared" si="0"/>
+        <v>1110</v>
+      </c>
+      <c r="J42" s="18">
+        <f t="shared" si="1"/>
+        <v>330</v>
+      </c>
+      <c r="K42" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L42" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M42" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N42" s="20" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="43" spans="1:14">
-      <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="14"/>
-      <c r="M43" s="14"/>
-      <c r="N43" s="15"/>
+      <c r="A43" s="16">
+        <v>46280</v>
+      </c>
+      <c r="B43" s="17">
+        <v>420</v>
+      </c>
+      <c r="C43" s="17">
+        <v>20</v>
+      </c>
+      <c r="D43" s="17">
+        <v>180</v>
+      </c>
+      <c r="E43" s="17">
+        <v>30</v>
+      </c>
+      <c r="F43" s="17">
+        <v>300</v>
+      </c>
+      <c r="G43" s="17">
+        <v>6</v>
+      </c>
+      <c r="H43" s="17">
+        <v>30</v>
+      </c>
+      <c r="I43" s="18">
+        <f t="shared" si="0"/>
+        <v>980</v>
+      </c>
+      <c r="J43" s="18">
+        <f t="shared" si="1"/>
+        <v>460</v>
+      </c>
+      <c r="K43" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L43" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M43" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="N43" s="20" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="44" spans="1:14">
-      <c r="A44" s="11"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="13"/>
-      <c r="J44" s="13"/>
-      <c r="K44" s="14"/>
-      <c r="L44" s="14"/>
-      <c r="M44" s="14"/>
-      <c r="N44" s="15"/>
+      <c r="A44" s="16">
+        <v>46281</v>
+      </c>
+      <c r="B44" s="17">
+        <v>420</v>
+      </c>
+      <c r="C44" s="17">
+        <v>20</v>
+      </c>
+      <c r="D44" s="17">
+        <v>180</v>
+      </c>
+      <c r="E44" s="17">
+        <v>40</v>
+      </c>
+      <c r="F44" s="17">
+        <v>300</v>
+      </c>
+      <c r="G44" s="17">
+        <v>6</v>
+      </c>
+      <c r="H44" s="17">
+        <v>20</v>
+      </c>
+      <c r="I44" s="18">
+        <f t="shared" si="0"/>
+        <v>980</v>
+      </c>
+      <c r="J44" s="18">
+        <f t="shared" si="1"/>
+        <v>460</v>
+      </c>
+      <c r="K44" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="L44" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M44" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="N44" s="20" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="45" spans="1:14">
-      <c r="A45" s="11"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="13" t="str">
+      <c r="A45" s="11">
+        <v>46282</v>
+      </c>
+      <c r="B45" s="12">
+        <v>420</v>
+      </c>
+      <c r="C45" s="12">
+        <v>20</v>
+      </c>
+      <c r="D45" s="12">
+        <v>180</v>
+      </c>
+      <c r="E45" s="12">
+        <v>60</v>
+      </c>
+      <c r="F45" s="12">
+        <v>200</v>
+      </c>
+      <c r="G45" s="12">
+        <v>4</v>
+      </c>
+      <c r="H45" s="12">
+        <v>30</v>
+      </c>
+      <c r="I45" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="13" t="str">
+        <v>910</v>
+      </c>
+      <c r="J45" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="14"/>
-      <c r="L45" s="14"/>
-      <c r="M45" s="14"/>
-      <c r="N45" s="15"/>
+        <v>530</v>
+      </c>
+      <c r="K45" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="L45" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="M45" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="N45" s="15" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="46" spans="1:14">
-      <c r="A46" s="11"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="13" t="str">
+      <c r="A46" s="11">
+        <v>46283</v>
+      </c>
+      <c r="B46" s="12">
+        <v>420</v>
+      </c>
+      <c r="C46" s="12">
+        <v>20</v>
+      </c>
+      <c r="D46" s="12">
+        <v>240</v>
+      </c>
+      <c r="E46" s="12">
+        <v>30</v>
+      </c>
+      <c r="F46" s="12">
+        <v>250</v>
+      </c>
+      <c r="G46" s="12">
+        <v>5</v>
+      </c>
+      <c r="H46" s="12">
+        <v>20</v>
+      </c>
+      <c r="I46" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="13" t="str">
+        <v>980</v>
+      </c>
+      <c r="J46" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-      <c r="N46" s="15"/>
-    </row>
-    <row r="47" spans="1:14">
-      <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="13" t="str">
+        <v>460</v>
+      </c>
+      <c r="K46" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="L46" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="M46" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="N46" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" ht="45" spans="1:14">
+      <c r="A47" s="11">
+        <v>46284</v>
+      </c>
+      <c r="B47" s="12">
+        <v>240</v>
+      </c>
+      <c r="C47" s="12">
+        <v>10</v>
+      </c>
+      <c r="D47" s="12">
+        <v>300</v>
+      </c>
+      <c r="E47" s="12">
+        <v>120</v>
+      </c>
+      <c r="F47" s="12">
+        <v>0</v>
+      </c>
+      <c r="G47" s="12">
+        <v>0</v>
+      </c>
+      <c r="H47" s="12">
+        <v>20</v>
+      </c>
+      <c r="I47" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="13" t="str">
+        <v>690</v>
+      </c>
+      <c r="J47" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="14"/>
-      <c r="L47" s="14"/>
-      <c r="M47" s="14"/>
-      <c r="N47" s="15"/>
+        <v>750</v>
+      </c>
+      <c r="K47" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="L47" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="M47" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="N47" s="15" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="11"/>
@@ -10850,19 +11472,24 @@
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="A4:N4"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J401">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+  <conditionalFormatting sqref="J29:J44">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:J28 J45:J401">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K401">
+    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K28 K29:K44 K45:K401">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L401">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L28 L29:L44 L45:L401">
       <formula1>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M401">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M28 M29:M44 M45:M401">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>